<commit_message>
SPM-93 Date the test cases 2026-10-09
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-93_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-93_Test_Cases.xlsx
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -1647,7 +1647,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -2649,7 +2649,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -2814,7 +2814,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -2978,7 +2978,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Written before the code (TDD, 2026-10-08), then built to them on 2026-10-08: every label, message and page address in the cases is what the code shows (checked against the screens' automated tests, not yet walked through by hand). Checked against the Week 1 briefing, Week 4 instructions, Week 7 Customer Changes and the discussion logs up to 20261006 (#124-#129). Entries marked DECIDED were chosen by the team rather than taken from the story; change them in code and cases together.</t>
+          <t>Written before the code (TDD, 2026-10-09), then built to them on 2026-10-09: every label, message and page address in the cases is what the code shows (checked against the screens' automated tests, not yet walked through by hand). Checked against the Week 1 briefing, Week 4 instructions, Week 7 Customer Changes and the discussion logs up to 20261006 (#124-#129). Entries marked DECIDED were chosen by the team rather than taken from the story; change them in code and cases together.</t>
         </is>
       </c>
       <c r="C2" s="11" t="n"/>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-08: the request page (S-15, 'Request a venue booking') replaces the AM/PM/Night checkboxes with 'Date', 'Start time' and 'End time' fields (one date per request, as before). The time fields accept any minute, so an off-grid time reaches the page's own check and its message rather than the browser's. Under them: 'Setup: HH:MM–HH:MM (N min)', 'Turnaround: HH:MM–HH:MM (N min)' and 'Room in use: HH:MM–HH:MM', or 'No setup or turnaround needed at this venue.' and 'Room in use: …' when both are zero.</t>
+          <t>DECIDED 2026-10-09: the request page (S-15, 'Request a venue booking') replaces the AM/PM/Night checkboxes with 'Date', 'Start time' and 'End time' fields (one date per request, as before). The time fields accept any minute, so an off-grid time reaches the page's own check and its message rather than the browser's. Under them: 'Setup: HH:MM–HH:MM (N min)', 'Turnaround: HH:MM–HH:MM (N min)' and 'Room in use: HH:MM–HH:MM', or 'No setup or turnaround needed at this venue.' and 'Room in use: …' when both are zero.</t>
         </is>
       </c>
       <c r="C3" s="11" t="n"/>
@@ -3094,7 +3094,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-08: refusal messages (AC3). Shown under the field: 'Choose a start time on a 15-minute step (:00, :15, :30 or :45).', 'Choose an end time on a 15-minute step (:00, :15, :30 or :45).', 'The end time must be after the start time.' The server applies the same checks.</t>
+          <t>DECIDED 2026-10-09: refusal messages (AC3). Shown under the field: 'Choose a start time on a 15-minute step (:00, :15, :30 or :45).', 'Choose an end time on a 15-minute step (:00, :15, :30 or :45).', 'The end time must be after the start time.' The server applies the same checks.</t>
         </is>
       </c>
       <c r="C4" s="11" t="n"/>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-08: the SPM-42 rule that the request must cover the event's (or session's) own time is kept, reworded 'The requested times do not cover the event's time (&lt;date&gt;, &lt;times&gt;).' ('session's' for a session).</t>
+          <t>DECIDED 2026-10-09: the SPM-42 rule that the request must cover the event's (or session's) own time is kept, reworded 'The requested times do not cover the event's time (&lt;date&gt;, &lt;times&gt;).' ('session's' for a session).</t>
         </is>
       </c>
       <c r="C5" s="11" t="n"/>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-08 (AC4, AC6): the whole room-in-use period, setup and turnaround included, must fit within the venue's opening hours, at request time and in Find a venue. Refusal: '&lt;venue&gt; is open 07:00–22:00. With its &lt;n&gt; min setup and &lt;n&gt; min turnaround, choose times between &lt;earliest start&gt; and &lt;latest end&gt;.' Not stated outright; inferred from Week 1 briefing (venue suitability depends on 'operating hours, setup requirements, and the turnaround time'), Week 7 Change #1 (setup and turnaround are when the venue is 'effectively occupied' and 'must be included when checking availability') and #46 (Venue Staff maintain operating hours). Our own question #131 (Q3, hours a venue can be booked) is still unanswered on 2026-10-08; if the customer rules otherwise, that ruling wins.</t>
+          <t>DECIDED 2026-10-09 (AC4, AC6): the whole room-in-use period, setup and turnaround included, must fit within the venue's opening hours, at request time and in Find a venue. Refusal: '&lt;venue&gt; is open 07:00–22:00. With its &lt;n&gt; min setup and &lt;n&gt; min turnaround, choose times between &lt;earliest start&gt; and &lt;latest end&gt;.' Not stated outright; inferred from Week 1 briefing (venue suitability depends on 'operating hours, setup requirements, and the turnaround time'), Week 7 Change #1 (setup and turnaround are when the venue is 'effectively occupied' and 'must be included when checking availability') and #46 (Venue Staff maintain operating hours). Our own question #131 (Q3, hours a venue can be booked) is still unanswered on 2026-10-09; if the customer rules otherwise, that ruling wins.</t>
         </is>
       </c>
       <c r="C6" s="11" t="n"/>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-09: refusals follow SPM-44 (Detect Venue Booking Conflicts, merged to main 2026-10-08), which names what is in the way (its AC9), with SPM-93's times in place of slots. At request time: '&lt;venue&gt; is already booked for &lt;reference&gt; &lt;title&gt; on &lt;date&gt;, &lt;from&gt;–&lt;to&gt;.' and '&lt;venue&gt; is on hold for &lt;reference&gt; &lt;title&gt; on &lt;date&gt;, &lt;from&gt;–&lt;to&gt;.', where the times are the minutes both need; '&lt;venue&gt; is unavailable at this time (&lt;reason&gt;, &lt;the period's own times&gt;).'; a repeat of the same request: 'This event already has a pending request for &lt;venue&gt; on &lt;date&gt;, &lt;times&gt;.' At approval: 'This overlaps an approved booking: &lt;reference&gt; &lt;title&gt; holds &lt;venue&gt; on &lt;date&gt;, &lt;times&gt; (room in use &lt;times&gt;).' plus ' The clash is through setup or turnaround time.' when the event times themselves do not overlap.</t>
+          <t>DECIDED 2026-10-09: refusals follow SPM-44 (Detect Venue Booking Conflicts, merged to main 2026-10-09), which names what is in the way (its AC9), with SPM-93's times in place of slots. At request time: '&lt;venue&gt; is already booked for &lt;reference&gt; &lt;title&gt; on &lt;date&gt;, &lt;from&gt;–&lt;to&gt;.' and '&lt;venue&gt; is on hold for &lt;reference&gt; &lt;title&gt; on &lt;date&gt;, &lt;from&gt;–&lt;to&gt;.', where the times are the minutes both need; '&lt;venue&gt; is unavailable at this time (&lt;reason&gt;, &lt;the period's own times&gt;).'; a repeat of the same request: 'This event already has a pending request for &lt;venue&gt; on &lt;date&gt;, &lt;times&gt;.' At approval: 'This overlaps an approved booking: &lt;reference&gt; &lt;title&gt; holds &lt;venue&gt; on &lt;date&gt;, &lt;times&gt; (room in use &lt;times&gt;).' plus ' The clash is through setup or turnaround time.' when the event times themselves do not overlap.</t>
         </is>
       </c>
       <c r="C7" s="11" t="n"/>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-08: on Booking Requests (S-22) the 'Requested' row shows '&lt;date&gt;, &lt;start&gt;–&lt;end&gt;' with the Setup, Turnaround and Room in use lines underneath (AC8). The approve dialog reads 'This books &lt;venue&gt; for &lt;reference&gt; &lt;title&gt; on &lt;date&gt;, &lt;times&gt;. No other event can then be booked into the room from &lt;start&gt; to &lt;end&gt;, which includes its setup and turnaround time.' The event's Venue tab shows each request as '&lt;date&gt;, &lt;start&gt;–&lt;end&gt; · &lt;layout&gt;'.</t>
+          <t>DECIDED 2026-10-09: on Booking Requests (S-22) the 'Requested' row shows '&lt;date&gt;, &lt;start&gt;–&lt;end&gt;' with the Setup, Turnaround and Room in use lines underneath (AC8). The approve dialog reads 'This books &lt;venue&gt; for &lt;reference&gt; &lt;title&gt; on &lt;date&gt;, &lt;times&gt;. No other event can then be booked into the room from &lt;start&gt; to &lt;end&gt;, which includes its setup and turnaround time.' The event's Venue tab shows each request as '&lt;date&gt;, &lt;start&gt;–&lt;end&gt; · &lt;layout&gt;'.</t>
         </is>
       </c>
       <c r="C8" s="11" t="n"/>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-08: venue form labels become 'Setup time (minutes)' and 'Turnaround time (minutes)' (the customer's word; the database field stays teardownMinutes). Hint 'In 15-minute steps: 0, 15, 30, 45 and so on.' Error 'Enter minutes in 15-minute steps: 0, 15, 30, 45 and so on.' The existing 'Enter a whole number of minutes, 0 or more.' still covers negative and non-numeric values. The calendar subtitle says 'turnaround' instead of 'teardown'. Week 7 Change #1 names only 'setup time' and 'turnaround time'; #43's 'teardown' is the same period.</t>
+          <t>DECIDED 2026-10-09: venue form labels become 'Setup time (minutes)' and 'Turnaround time (minutes)' (the customer's word; the database field stays teardownMinutes). Hint 'In 15-minute steps: 0, 15, 30, 45 and so on.' Error 'Enter minutes in 15-minute steps: 0, 15, 30, 45 and so on.' The existing 'Enter a whole number of minutes, 0 or more.' still covers negative and non-numeric values. The calendar subtitle says 'turnaround' instead of 'teardown'. Week 7 Change #1 names only 'setup time' and 'turnaround time'; #43's 'teardown' is the same period.</t>
         </is>
       </c>
       <c r="C9" s="11" t="n"/>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-08 (AC9): the availability calendar (S-21) keeps one row per day but replaces the AM/PM/Night columns with one 'Schedule' column. Each entry reads '&lt;kind&gt; HH:MM–HH:MM · &lt;event title or reason&gt;', in time order, where kind is 'Setup', 'Booked', 'Turnaround', 'Requested' (a pending hold) or 'Unavailable'. An empty day shows 'Free' ('Closed' for a retired venue). The Unavailable periods card shows times, not just dates. The warning about minutes 'outside the AM, PM and Night slots' is removed. Layout is ours to choose: #6 says calendar granularity 'is a UI/UX question, please propose'.</t>
+          <t>DECIDED 2026-10-09 (AC9): the availability calendar (S-21) keeps one row per day but replaces the AM/PM/Night columns with one 'Schedule' column. Each entry reads '&lt;kind&gt; HH:MM–HH:MM · &lt;event title or reason&gt;', in time order, where kind is 'Setup', 'Booked', 'Turnaround', 'Requested' (a pending hold) or 'Unavailable'. An empty day shows 'Free' ('Closed' for a retired venue). The Unavailable periods card shows times, not just dates. The warning about minutes 'outside the AM, PM and Night slots' is removed. Layout is ours to choose: #6 says calendar granularity 'is a UI/UX question, please propose'.</t>
         </is>
       </c>
       <c r="C10" s="11" t="n"/>
@@ -3301,7 +3301,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -3643,7 +3643,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -3808,7 +3808,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -3979,7 +3979,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -4151,7 +4151,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">
@@ -4318,7 +4318,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
SPM-93 Date every test case and note 2026-10-08, when they were written
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-93_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-93_Test_Cases.xlsx
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -1647,7 +1647,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -2315,7 +2315,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -2649,7 +2649,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -2814,7 +2814,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -2978,7 +2978,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Written before the code (TDD, 2026-10-09), then built to them on 2026-10-09: every label, message and page address in the cases is what the code shows (checked against the screens' automated tests, not yet walked through by hand). Checked against the Week 1 briefing, Week 4 instructions, Week 7 Customer Changes and the discussion logs up to 20261006 (#124-#129). Entries marked DECIDED were chosen by the team rather than taken from the story; change them in code and cases together.</t>
+          <t>Written before the code (TDD, 2026-10-08), then built to them on 2026-10-08: every label, message and page address in the cases is what the code shows (checked against the screens' automated tests, not yet walked through by hand). Checked against the Week 1 briefing, Week 4 instructions, Week 7 Customer Changes and the discussion logs up to 20261006 (#124-#129). Entries marked DECIDED were chosen by the team rather than taken from the story; change them in code and cases together.</t>
         </is>
       </c>
       <c r="C2" s="11" t="n"/>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-09: the request page (S-15, 'Request a venue booking') replaces the AM/PM/Night checkboxes with 'Date', 'Start time' and 'End time' fields (one date per request, as before). The time fields accept any minute, so an off-grid time reaches the page's own check and its message rather than the browser's. Under them: 'Setup: HH:MM–HH:MM (N min)', 'Turnaround: HH:MM–HH:MM (N min)' and 'Room in use: HH:MM–HH:MM', or 'No setup or turnaround needed at this venue.' and 'Room in use: …' when both are zero.</t>
+          <t>DECIDED 2026-10-08: the request page (S-15, 'Request a venue booking') replaces the AM/PM/Night checkboxes with 'Date', 'Start time' and 'End time' fields (one date per request, as before). The time fields accept any minute, so an off-grid time reaches the page's own check and its message rather than the browser's. Under them: 'Setup: HH:MM–HH:MM (N min)', 'Turnaround: HH:MM–HH:MM (N min)' and 'Room in use: HH:MM–HH:MM', or 'No setup or turnaround needed at this venue.' and 'Room in use: …' when both are zero.</t>
         </is>
       </c>
       <c r="C3" s="11" t="n"/>
@@ -3094,7 +3094,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-09: refusal messages (AC3). Shown under the field: 'Choose a start time on a 15-minute step (:00, :15, :30 or :45).', 'Choose an end time on a 15-minute step (:00, :15, :30 or :45).', 'The end time must be after the start time.' The server applies the same checks.</t>
+          <t>DECIDED 2026-10-08: refusal messages (AC3). Shown under the field: 'Choose a start time on a 15-minute step (:00, :15, :30 or :45).', 'Choose an end time on a 15-minute step (:00, :15, :30 or :45).', 'The end time must be after the start time.' The server applies the same checks.</t>
         </is>
       </c>
       <c r="C4" s="11" t="n"/>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-09: the SPM-42 rule that the request must cover the event's (or session's) own time is kept, reworded 'The requested times do not cover the event's time (&lt;date&gt;, &lt;times&gt;).' ('session's' for a session).</t>
+          <t>DECIDED 2026-10-08: the SPM-42 rule that the request must cover the event's (or session's) own time is kept, reworded 'The requested times do not cover the event's time (&lt;date&gt;, &lt;times&gt;).' ('session's' for a session).</t>
         </is>
       </c>
       <c r="C5" s="11" t="n"/>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-09 (AC4, AC6): the whole room-in-use period, setup and turnaround included, must fit within the venue's opening hours, at request time and in Find a venue. Refusal: '&lt;venue&gt; is open 07:00–22:00. With its &lt;n&gt; min setup and &lt;n&gt; min turnaround, choose times between &lt;earliest start&gt; and &lt;latest end&gt;.' Not stated outright; inferred from Week 1 briefing (venue suitability depends on 'operating hours, setup requirements, and the turnaround time'), Week 7 Change #1 (setup and turnaround are when the venue is 'effectively occupied' and 'must be included when checking availability') and #46 (Venue Staff maintain operating hours). Our own question #131 (Q3, hours a venue can be booked) is still unanswered on 2026-10-09; if the customer rules otherwise, that ruling wins.</t>
+          <t>DECIDED 2026-10-08 (AC4, AC6): the whole room-in-use period, setup and turnaround included, must fit within the venue's opening hours, at request time and in Find a venue. Refusal: '&lt;venue&gt; is open 07:00–22:00. With its &lt;n&gt; min setup and &lt;n&gt; min turnaround, choose times between &lt;earliest start&gt; and &lt;latest end&gt;.' Not stated outright; inferred from Week 1 briefing (venue suitability depends on 'operating hours, setup requirements, and the turnaround time'), Week 7 Change #1 (setup and turnaround are when the venue is 'effectively occupied' and 'must be included when checking availability') and #46 (Venue Staff maintain operating hours). Our own question #131 (Q3, hours a venue can be booked) is still unanswered on 2026-10-08; if the customer rules otherwise, that ruling wins.</t>
         </is>
       </c>
       <c r="C6" s="11" t="n"/>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-09: refusals follow SPM-44 (Detect Venue Booking Conflicts, merged to main 2026-10-09), which names what is in the way (its AC9), with SPM-93's times in place of slots. At request time: '&lt;venue&gt; is already booked for &lt;reference&gt; &lt;title&gt; on &lt;date&gt;, &lt;from&gt;–&lt;to&gt;.' and '&lt;venue&gt; is on hold for &lt;reference&gt; &lt;title&gt; on &lt;date&gt;, &lt;from&gt;–&lt;to&gt;.', where the times are the minutes both need; '&lt;venue&gt; is unavailable at this time (&lt;reason&gt;, &lt;the period's own times&gt;).'; a repeat of the same request: 'This event already has a pending request for &lt;venue&gt; on &lt;date&gt;, &lt;times&gt;.' At approval: 'This overlaps an approved booking: &lt;reference&gt; &lt;title&gt; holds &lt;venue&gt; on &lt;date&gt;, &lt;times&gt; (room in use &lt;times&gt;).' plus ' The clash is through setup or turnaround time.' when the event times themselves do not overlap.</t>
+          <t>DECIDED 2026-10-08: refusals follow SPM-44 (Detect Venue Booking Conflicts, merged to main 2026-10-08), which names what is in the way (its AC9), with SPM-93's times in place of slots. At request time: '&lt;venue&gt; is already booked for &lt;reference&gt; &lt;title&gt; on &lt;date&gt;, &lt;from&gt;–&lt;to&gt;.' and '&lt;venue&gt; is on hold for &lt;reference&gt; &lt;title&gt; on &lt;date&gt;, &lt;from&gt;–&lt;to&gt;.', where the times are the minutes both need; '&lt;venue&gt; is unavailable at this time (&lt;reason&gt;, &lt;the period's own times&gt;).'; a repeat of the same request: 'This event already has a pending request for &lt;venue&gt; on &lt;date&gt;, &lt;times&gt;.' At approval: 'This overlaps an approved booking: &lt;reference&gt; &lt;title&gt; holds &lt;venue&gt; on &lt;date&gt;, &lt;times&gt; (room in use &lt;times&gt;).' plus ' The clash is through setup or turnaround time.' when the event times themselves do not overlap.</t>
         </is>
       </c>
       <c r="C7" s="11" t="n"/>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-09: on Booking Requests (S-22) the 'Requested' row shows '&lt;date&gt;, &lt;start&gt;–&lt;end&gt;' with the Setup, Turnaround and Room in use lines underneath (AC8). The approve dialog reads 'This books &lt;venue&gt; for &lt;reference&gt; &lt;title&gt; on &lt;date&gt;, &lt;times&gt;. No other event can then be booked into the room from &lt;start&gt; to &lt;end&gt;, which includes its setup and turnaround time.' The event's Venue tab shows each request as '&lt;date&gt;, &lt;start&gt;–&lt;end&gt; · &lt;layout&gt;'.</t>
+          <t>DECIDED 2026-10-08: on Booking Requests (S-22) the 'Requested' row shows '&lt;date&gt;, &lt;start&gt;–&lt;end&gt;' with the Setup, Turnaround and Room in use lines underneath (AC8). The approve dialog reads 'This books &lt;venue&gt; for &lt;reference&gt; &lt;title&gt; on &lt;date&gt;, &lt;times&gt;. No other event can then be booked into the room from &lt;start&gt; to &lt;end&gt;, which includes its setup and turnaround time.' The event's Venue tab shows each request as '&lt;date&gt;, &lt;start&gt;–&lt;end&gt; · &lt;layout&gt;'.</t>
         </is>
       </c>
       <c r="C8" s="11" t="n"/>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-09: venue form labels become 'Setup time (minutes)' and 'Turnaround time (minutes)' (the customer's word; the database field stays teardownMinutes). Hint 'In 15-minute steps: 0, 15, 30, 45 and so on.' Error 'Enter minutes in 15-minute steps: 0, 15, 30, 45 and so on.' The existing 'Enter a whole number of minutes, 0 or more.' still covers negative and non-numeric values. The calendar subtitle says 'turnaround' instead of 'teardown'. Week 7 Change #1 names only 'setup time' and 'turnaround time'; #43's 'teardown' is the same period.</t>
+          <t>DECIDED 2026-10-08: venue form labels become 'Setup time (minutes)' and 'Turnaround time (minutes)' (the customer's word; the database field stays teardownMinutes). Hint 'In 15-minute steps: 0, 15, 30, 45 and so on.' Error 'Enter minutes in 15-minute steps: 0, 15, 30, 45 and so on.' The existing 'Enter a whole number of minutes, 0 or more.' still covers negative and non-numeric values. The calendar subtitle says 'turnaround' instead of 'teardown'. Week 7 Change #1 names only 'setup time' and 'turnaround time'; #43's 'teardown' is the same period.</t>
         </is>
       </c>
       <c r="C9" s="11" t="n"/>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-09 (AC9): the availability calendar (S-21) keeps one row per day but replaces the AM/PM/Night columns with one 'Schedule' column. Each entry reads '&lt;kind&gt; HH:MM–HH:MM · &lt;event title or reason&gt;', in time order, where kind is 'Setup', 'Booked', 'Turnaround', 'Requested' (a pending hold) or 'Unavailable'. An empty day shows 'Free' ('Closed' for a retired venue). The Unavailable periods card shows times, not just dates. The warning about minutes 'outside the AM, PM and Night slots' is removed. Layout is ours to choose: #6 says calendar granularity 'is a UI/UX question, please propose'.</t>
+          <t>DECIDED 2026-10-08 (AC9): the availability calendar (S-21) keeps one row per day but replaces the AM/PM/Night columns with one 'Schedule' column. Each entry reads '&lt;kind&gt; HH:MM–HH:MM · &lt;event title or reason&gt;', in time order, where kind is 'Setup', 'Booked', 'Turnaround', 'Requested' (a pending hold) or 'Unavailable'. An empty day shows 'Free' ('Closed' for a retired venue). The Unavailable periods card shows times, not just dates. The warning about minutes 'outside the AM, PM and Night slots' is removed. Layout is ours to choose: #6 says calendar granularity 'is a UI/UX question, please propose'.</t>
         </is>
       </c>
       <c r="C10" s="11" t="n"/>
@@ -3301,7 +3301,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -3643,7 +3643,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -3808,7 +3808,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -3979,7 +3979,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -4151,7 +4151,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">
@@ -4318,7 +4318,7 @@
         </is>
       </c>
       <c r="B8" s="14" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="10">

</xml_diff>